<commit_message>
feat: calibrate new alliance-zone07 lightbar
</commit_message>
<xml_diff>
--- a/scripts/calibration/Plant Chamber Full Calibration.xlsx
+++ b/scripts/calibration/Plant Chamber Full Calibration.xlsx
@@ -3,18 +3,19 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="zone01" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="zone02" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="zone03" sheetId="3" r:id="rId6"/>
-    <sheet state="visible" name="zone04" sheetId="4" r:id="rId7"/>
-    <sheet state="visible" name="zone05" sheetId="5" r:id="rId8"/>
-    <sheet state="visible" name="zone06" sheetId="6" r:id="rId9"/>
-    <sheet state="visible" name="zone07" sheetId="7" r:id="rId10"/>
-    <sheet state="visible" name="zone08" sheetId="8" r:id="rId11"/>
-    <sheet state="visible" name="zone09" sheetId="9" r:id="rId12"/>
-    <sheet state="visible" name="zone10" sheetId="10" r:id="rId13"/>
-    <sheet state="visible" name="zone11" sheetId="11" r:id="rId14"/>
-    <sheet state="visible" name="zone12" sheetId="12" r:id="rId15"/>
+    <sheet state="visible" name="zone01" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="zone02" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="zone03" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="zone04" sheetId="4" r:id="rId8"/>
+    <sheet state="visible" name="zone05" sheetId="5" r:id="rId9"/>
+    <sheet state="visible" name="zone06" sheetId="6" r:id="rId10"/>
+    <sheet state="visible" name="zone07" sheetId="7" r:id="rId11"/>
+    <sheet state="visible" name="zone08" sheetId="8" r:id="rId12"/>
+    <sheet state="visible" name="zone09" sheetId="9" r:id="rId13"/>
+    <sheet state="visible" name="zone10" sheetId="10" r:id="rId14"/>
+    <sheet state="visible" name="zone11" sheetId="11" r:id="rId15"/>
+    <sheet state="visible" name="zone12" sheetId="12" r:id="rId16"/>
+    <sheet state="visible" name="Sheet3" sheetId="13" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="6">
   <si>
     <t>Action</t>
   </si>
@@ -80,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -99,6 +100,21 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="2" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="2" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="2" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -297,11 +313,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="2080668723"/>
-        <c:axId val="262435632"/>
+        <c:axId val="429170077"/>
+        <c:axId val="1713102312"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="2080668723"/>
+        <c:axId val="429170077"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -353,10 +369,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="262435632"/>
+        <c:crossAx val="1713102312"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="262435632"/>
+        <c:axId val="1713102312"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -431,7 +447,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2080668723"/>
+        <c:crossAx val="429170077"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -646,11 +662,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="2113415182"/>
-        <c:axId val="991111995"/>
+        <c:axId val="16475450"/>
+        <c:axId val="448111536"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="2113415182"/>
+        <c:axId val="16475450"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -702,10 +718,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="991111995"/>
+        <c:crossAx val="448111536"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="991111995"/>
+        <c:axId val="448111536"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -780,7 +796,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2113415182"/>
+        <c:crossAx val="16475450"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -995,11 +1011,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1707158049"/>
-        <c:axId val="1220524161"/>
+        <c:axId val="970120161"/>
+        <c:axId val="1765628906"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1707158049"/>
+        <c:axId val="970120161"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1051,10 +1067,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1220524161"/>
+        <c:crossAx val="1765628906"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1220524161"/>
+        <c:axId val="1765628906"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1129,7 +1145,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1707158049"/>
+        <c:crossAx val="970120161"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1344,11 +1360,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1747378314"/>
-        <c:axId val="991459655"/>
+        <c:axId val="138516305"/>
+        <c:axId val="1209531658"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1747378314"/>
+        <c:axId val="138516305"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1400,10 +1416,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="991459655"/>
+        <c:crossAx val="1209531658"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="991459655"/>
+        <c:axId val="1209531658"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1478,7 +1494,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1747378314"/>
+        <c:crossAx val="138516305"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1504,7 +1520,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart13.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
   <c:chart>
     <c:title>
@@ -1528,7 +1544,7 @@
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
               </a:rPr>
-              <a:t>Blue, Cool_white, warm_white, orange_red, red…</a:t>
+              <a:t>Red vs. Action</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1538,12 +1554,13 @@
     <c:plotArea>
       <c:layout/>
       <c:lineChart>
+        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>zone02!$A$2</c:f>
+              <c:f>Sheet3!$A$1</c:f>
             </c:strRef>
           </c:tx>
           <c:spPr>
@@ -1558,146 +1575,22 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>zone02!$B$1:$O$1</c:f>
+              <c:f>Sheet3!$B$2:$B$14</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>zone02!$B$2:$O$2</c:f>
+              <c:f>Sheet3!$A$2:$A$14</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>zone02!$A$3</c:f>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln cmpd="sng">
-              <a:solidFill>
-                <a:srgbClr val="EA4335"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>zone02!$B$1:$O$1</c:f>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>zone02!$B$3:$O$3</c:f>
-              <c:numCache/>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>zone02!$A$4</c:f>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln cmpd="sng">
-              <a:solidFill>
-                <a:srgbClr val="FBBC04"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>zone02!$B$1:$O$1</c:f>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>zone02!$B$4:$O$4</c:f>
-              <c:numCache/>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-        </c:ser>
-        <c:ser>
-          <c:idx val="3"/>
-          <c:order val="3"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>zone02!$A$5</c:f>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln cmpd="sng">
-              <a:solidFill>
-                <a:srgbClr val="34A853"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>zone02!$B$1:$O$1</c:f>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>zone02!$B$5:$O$5</c:f>
-              <c:numCache/>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-        </c:ser>
-        <c:ser>
-          <c:idx val="4"/>
-          <c:order val="4"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>zone02!$A$6</c:f>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln cmpd="sng">
-              <a:solidFill>
-                <a:srgbClr val="FF6D01"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>zone02!$B$1:$O$1</c:f>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>zone02!$B$6:$O$6</c:f>
-              <c:numCache/>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-        </c:ser>
-        <c:axId val="599727006"/>
-        <c:axId val="685455045"/>
+        <c:axId val="1130418289"/>
+        <c:axId val="62630985"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="599727006"/>
+        <c:axId val="1130418289"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1749,10 +1642,359 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="685455045"/>
+        <c:crossAx val="62630985"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="685455045"/>
+        <c:axId val="62630985"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC">
+                  <a:alpha val="0"/>
+                </a:srgbClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:rPr>
+                  <a:t>Red</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1130418289"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr b="0">
+              <a:solidFill>
+                <a:srgbClr val="1A1A1A"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="757575"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="757575"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:rPr>
+              <a:t>Blue, Cool_white, warm_white, orange_red, red…</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>zone02!$A$2</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="4285F4"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>zone02!$B$1:$O$1</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>zone02!$B$2:$O$2</c:f>
+              <c:numCache/>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>zone02!$A$3</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="EA4335"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>zone02!$B$1:$O$1</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>zone02!$B$3:$O$3</c:f>
+              <c:numCache/>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>zone02!$A$4</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="FBBC04"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>zone02!$B$1:$O$1</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>zone02!$B$4:$O$4</c:f>
+              <c:numCache/>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>zone02!$A$5</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="34A853"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>zone02!$B$1:$O$1</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>zone02!$B$5:$O$5</c:f>
+              <c:numCache/>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>zone02!$A$6</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="FF6D01"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>zone02!$B$1:$O$1</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>zone02!$B$6:$O$6</c:f>
+              <c:numCache/>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:axId val="1749627864"/>
+        <c:axId val="19195572"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1749627864"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:rPr>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:spPr/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="19195572"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="19195572"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1827,7 +2069,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="599727006"/>
+        <c:crossAx val="1749627864"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2042,11 +2284,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="22438184"/>
-        <c:axId val="30076147"/>
+        <c:axId val="1843744859"/>
+        <c:axId val="1642447823"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="22438184"/>
+        <c:axId val="1843744859"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2098,10 +2340,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30076147"/>
+        <c:crossAx val="1642447823"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="30076147"/>
+        <c:axId val="1642447823"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2176,7 +2418,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22438184"/>
+        <c:crossAx val="1843744859"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2391,11 +2633,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="657546117"/>
-        <c:axId val="715258471"/>
+        <c:axId val="2022266646"/>
+        <c:axId val="371642799"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="657546117"/>
+        <c:axId val="2022266646"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2447,10 +2689,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="715258471"/>
+        <c:crossAx val="371642799"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="715258471"/>
+        <c:axId val="371642799"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2525,7 +2767,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="657546117"/>
+        <c:crossAx val="2022266646"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2740,11 +2982,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="563166438"/>
-        <c:axId val="695682241"/>
+        <c:axId val="1891774395"/>
+        <c:axId val="512140186"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="563166438"/>
+        <c:axId val="1891774395"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2796,10 +3038,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="695682241"/>
+        <c:crossAx val="512140186"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="695682241"/>
+        <c:axId val="512140186"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2874,7 +3116,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="563166438"/>
+        <c:crossAx val="1891774395"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -3089,11 +3331,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1820256411"/>
-        <c:axId val="361093923"/>
+        <c:axId val="1086680974"/>
+        <c:axId val="1182942974"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1820256411"/>
+        <c:axId val="1086680974"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3145,10 +3387,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="361093923"/>
+        <c:crossAx val="1182942974"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="361093923"/>
+        <c:axId val="1182942974"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3223,7 +3465,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1820256411"/>
+        <c:crossAx val="1086680974"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -3438,11 +3680,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="2043071111"/>
-        <c:axId val="1177543730"/>
+        <c:axId val="888574473"/>
+        <c:axId val="1708187801"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="2043071111"/>
+        <c:axId val="888574473"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3494,10 +3736,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1177543730"/>
+        <c:crossAx val="1708187801"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1177543730"/>
+        <c:axId val="1708187801"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3572,7 +3814,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2043071111"/>
+        <c:crossAx val="888574473"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -3787,11 +4029,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="2099023770"/>
-        <c:axId val="1091326507"/>
+        <c:axId val="115506843"/>
+        <c:axId val="999718733"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="2099023770"/>
+        <c:axId val="115506843"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3843,10 +4085,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1091326507"/>
+        <c:crossAx val="999718733"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1091326507"/>
+        <c:axId val="999718733"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3921,7 +4163,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2099023770"/>
+        <c:crossAx val="115506843"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -4136,11 +4378,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1586485899"/>
-        <c:axId val="490435914"/>
+        <c:axId val="1090802965"/>
+        <c:axId val="623656772"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1586485899"/>
+        <c:axId val="1090802965"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4192,10 +4434,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="490435914"/>
+        <c:crossAx val="623656772"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="490435914"/>
+        <c:axId val="623656772"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4270,7 +4512,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1586485899"/>
+        <c:crossAx val="1090802965"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -4399,6 +4641,36 @@
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="12" name="Chart 12" title="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>200025</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5715000" cy="3533775"/>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="13" name="Chart 13" title="Chart"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -4656,6 +4928,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
   <a:themeElements>
@@ -6068,6 +6344,184 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="9"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="7"/>
+      <c r="T1" s="7"/>
+      <c r="U1" s="7"/>
+      <c r="V1" s="7"/>
+      <c r="W1" s="7"/>
+      <c r="X1" s="7"/>
+      <c r="Y1" s="7"/>
+      <c r="Z1" s="7"/>
+      <c r="AA1" s="7"/>
+      <c r="AB1" s="7"/>
+      <c r="AC1" s="7"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="B2" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="11"/>
+      <c r="M2" s="11"/>
+      <c r="N2" s="11"/>
+      <c r="O2" s="8"/>
+      <c r="P2" s="8"/>
+      <c r="Q2" s="8"/>
+      <c r="R2" s="8"/>
+      <c r="S2" s="8"/>
+      <c r="T2" s="8"/>
+      <c r="U2" s="8"/>
+      <c r="V2" s="8"/>
+      <c r="W2" s="8"/>
+      <c r="X2" s="8"/>
+      <c r="Y2" s="8"/>
+      <c r="Z2" s="8"/>
+      <c r="AA2" s="8"/>
+      <c r="AB2" s="8"/>
+      <c r="AC2" s="8"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="B3" s="11">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10">
+        <v>0.3</v>
+      </c>
+      <c r="B4" s="11">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10">
+        <v>0.35</v>
+      </c>
+      <c r="B5" s="11">
+        <v>10.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10">
+        <v>0.4</v>
+      </c>
+      <c r="B6" s="11">
+        <v>16.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="B7" s="11">
+        <v>30.0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10">
+        <v>0.6</v>
+      </c>
+      <c r="B8" s="11">
+        <v>42.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10">
+        <v>0.7</v>
+      </c>
+      <c r="B9" s="11">
+        <v>54.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10">
+        <v>0.8</v>
+      </c>
+      <c r="B10" s="11">
+        <v>67.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10">
+        <v>0.85</v>
+      </c>
+      <c r="B11" s="11">
+        <v>71.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10">
+        <v>0.9</v>
+      </c>
+      <c r="B12" s="11">
+        <v>74.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10">
+        <v>0.95</v>
+      </c>
+      <c r="B13" s="11">
+        <v>75.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10">
+        <v>1.0</v>
+      </c>
+      <c r="B14" s="11">
+        <v>75.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
@@ -7669,40 +8123,40 @@
         <v>0.0</v>
       </c>
       <c r="C2" s="4">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D2" s="4">
-        <v>6.0</v>
+        <v>3.0</v>
       </c>
       <c r="E2" s="4">
-        <v>14.0</v>
+        <v>9.0</v>
       </c>
       <c r="F2" s="4">
-        <v>23.0</v>
+        <v>18.0</v>
       </c>
       <c r="G2" s="4">
-        <v>42.0</v>
+        <v>34.0</v>
       </c>
       <c r="H2" s="4">
-        <v>59.0</v>
+        <v>49.0</v>
       </c>
       <c r="I2" s="4">
-        <v>75.0</v>
+        <v>64.0</v>
       </c>
       <c r="J2" s="4">
+        <v>78.0</v>
+      </c>
+      <c r="K2" s="4">
+        <v>84.0</v>
+      </c>
+      <c r="L2" s="4">
         <v>91.0</v>
       </c>
-      <c r="K2" s="4">
-        <v>98.0</v>
-      </c>
-      <c r="L2" s="4">
-        <v>105.0</v>
-      </c>
       <c r="M2" s="4">
-        <v>111.0</v>
+        <v>96.0</v>
       </c>
       <c r="N2" s="4">
-        <v>114.0</v>
+        <v>100.0</v>
       </c>
     </row>
     <row r="3">
@@ -7713,40 +8167,40 @@
         <v>0.0</v>
       </c>
       <c r="C3" s="4">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D3" s="4">
-        <v>6.0</v>
+        <v>3.0</v>
       </c>
       <c r="E3" s="4">
-        <v>13.0</v>
+        <v>9.0</v>
       </c>
       <c r="F3" s="4">
-        <v>22.0</v>
+        <v>17.0</v>
       </c>
       <c r="G3" s="4">
-        <v>39.0</v>
+        <v>32.0</v>
       </c>
       <c r="H3" s="4">
-        <v>55.0</v>
+        <v>47.0</v>
       </c>
       <c r="I3" s="4">
-        <v>71.0</v>
+        <v>61.0</v>
       </c>
       <c r="J3" s="4">
-        <v>85.0</v>
+        <v>74.0</v>
       </c>
       <c r="K3" s="4">
-        <v>92.0</v>
+        <v>81.0</v>
       </c>
       <c r="L3" s="4">
-        <v>99.0</v>
+        <v>87.0</v>
       </c>
       <c r="M3" s="4">
-        <v>106.0</v>
+        <v>93.0</v>
       </c>
       <c r="N3" s="4">
-        <v>112.0</v>
+        <v>98.0</v>
       </c>
     </row>
     <row r="4">
@@ -7760,37 +8214,37 @@
         <v>0.0</v>
       </c>
       <c r="D4" s="4">
-        <v>5.0</v>
+        <v>3.0</v>
       </c>
       <c r="E4" s="4">
-        <v>11.0</v>
+        <v>8.0</v>
       </c>
       <c r="F4" s="4">
-        <v>18.0</v>
+        <v>14.0</v>
       </c>
       <c r="G4" s="4">
-        <v>33.0</v>
+        <v>28.0</v>
       </c>
       <c r="H4" s="4">
-        <v>45.0</v>
+        <v>40.0</v>
       </c>
       <c r="I4" s="4">
-        <v>59.0</v>
+        <v>51.0</v>
       </c>
       <c r="J4" s="4">
-        <v>70.0</v>
+        <v>62.0</v>
       </c>
       <c r="K4" s="4">
+        <v>67.0</v>
+      </c>
+      <c r="L4" s="4">
+        <v>72.0</v>
+      </c>
+      <c r="M4" s="4">
         <v>76.0</v>
       </c>
-      <c r="L4" s="4">
-        <v>81.0</v>
-      </c>
-      <c r="M4" s="4">
-        <v>87.0</v>
-      </c>
       <c r="N4" s="4">
-        <v>91.0</v>
+        <v>80.0</v>
       </c>
     </row>
     <row r="5">
@@ -7804,37 +8258,37 @@
         <v>1.0</v>
       </c>
       <c r="D5" s="4">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="E5" s="4">
-        <v>13.0</v>
+        <v>11.0</v>
       </c>
       <c r="F5" s="4">
-        <v>21.0</v>
+        <v>19.0</v>
       </c>
       <c r="G5" s="4">
-        <v>38.0</v>
+        <v>34.0</v>
       </c>
       <c r="H5" s="4">
-        <v>54.0</v>
+        <v>49.0</v>
       </c>
       <c r="I5" s="4">
-        <v>69.0</v>
+        <v>63.0</v>
       </c>
       <c r="J5" s="4">
-        <v>82.0</v>
+        <v>75.0</v>
       </c>
       <c r="K5" s="4">
-        <v>87.0</v>
+        <v>78.0</v>
       </c>
       <c r="L5" s="4">
-        <v>89.0</v>
+        <v>79.0</v>
       </c>
       <c r="M5" s="4">
-        <v>90.0</v>
+        <v>79.0</v>
       </c>
       <c r="N5" s="4">
-        <v>90.0</v>
+        <v>79.0</v>
       </c>
     </row>
     <row r="6">
@@ -7848,37 +8302,37 @@
         <v>0.0</v>
       </c>
       <c r="D6" s="4">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="E6" s="4">
-        <v>5.0</v>
+        <v>9.0</v>
       </c>
       <c r="F6" s="4">
-        <v>8.0</v>
+        <v>16.0</v>
       </c>
       <c r="G6" s="4">
-        <v>14.0</v>
+        <v>30.0</v>
       </c>
       <c r="H6" s="4">
-        <v>21.0</v>
+        <v>43.0</v>
       </c>
       <c r="I6" s="4">
-        <v>27.0</v>
+        <v>54.0</v>
       </c>
       <c r="J6" s="4">
-        <v>29.0</v>
+        <v>59.0</v>
       </c>
       <c r="K6" s="4">
-        <v>29.0</v>
+        <v>60.0</v>
       </c>
       <c r="L6" s="4">
-        <v>29.0</v>
+        <v>60.0</v>
       </c>
       <c r="M6" s="4">
-        <v>29.0</v>
+        <v>60.0</v>
       </c>
       <c r="N6" s="4">
-        <v>29.0</v>
+        <v>60.0</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
feat: re-calibrate zone 5
</commit_message>
<xml_diff>
--- a/scripts/calibration/Plant Chamber Full Calibration.xlsx
+++ b/scripts/calibration/Plant Chamber Full Calibration.xlsx
@@ -12,9 +12,9 @@
     <sheet state="visible" name="zone07" sheetId="7" r:id="rId11"/>
     <sheet state="visible" name="zone08" sheetId="8" r:id="rId12"/>
     <sheet state="visible" name="zone09" sheetId="9" r:id="rId13"/>
-    <sheet state="visible" name="zone10" sheetId="10" r:id="rId14"/>
+    <sheet state="visible" name="zone12" sheetId="10" r:id="rId14"/>
     <sheet state="visible" name="zone11" sheetId="11" r:id="rId15"/>
-    <sheet state="visible" name="zone12" sheetId="12" r:id="rId16"/>
+    <sheet state="visible" name="zone10" sheetId="12" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -297,11 +297,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1282783026"/>
-        <c:axId val="789588921"/>
+        <c:axId val="2108648301"/>
+        <c:axId val="1447308777"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1282783026"/>
+        <c:axId val="2108648301"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -338,7 +338,11 @@
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:spPr/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
@@ -353,10 +357,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="789588921"/>
+        <c:crossAx val="1447308777"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="789588921"/>
+        <c:axId val="1447308777"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -415,7 +419,9 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
-          <a:ln/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
         </c:spPr>
         <c:txPr>
           <a:bodyPr/>
@@ -431,7 +437,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1282783026"/>
+        <c:crossAx val="2108648301"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -496,7 +502,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>zone10!$A$2</c:f>
+              <c:f>zone12!$A$2</c:f>
             </c:strRef>
           </c:tx>
           <c:spPr>
@@ -511,12 +517,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>zone10!$B$1:$M$1</c:f>
+              <c:f>zone12!$B$1:$M$1</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>zone10!$B$2:$M$2</c:f>
+              <c:f>zone12!$B$2:$M$2</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -527,7 +533,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>zone10!$A$3</c:f>
+              <c:f>zone12!$A$3</c:f>
             </c:strRef>
           </c:tx>
           <c:spPr>
@@ -542,12 +548,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>zone10!$B$1:$M$1</c:f>
+              <c:f>zone12!$B$1:$M$1</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>zone10!$B$3:$M$3</c:f>
+              <c:f>zone12!$B$3:$M$3</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -558,7 +564,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>zone10!$A$4</c:f>
+              <c:f>zone12!$A$4</c:f>
             </c:strRef>
           </c:tx>
           <c:spPr>
@@ -573,12 +579,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>zone10!$B$1:$M$1</c:f>
+              <c:f>zone12!$B$1:$M$1</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>zone10!$B$4:$M$4</c:f>
+              <c:f>zone12!$B$4:$M$4</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -589,7 +595,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>zone10!$A$5</c:f>
+              <c:f>zone12!$A$5</c:f>
             </c:strRef>
           </c:tx>
           <c:spPr>
@@ -604,12 +610,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>zone10!$B$1:$M$1</c:f>
+              <c:f>zone12!$B$1:$M$1</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>zone10!$B$5:$M$5</c:f>
+              <c:f>zone12!$B$5:$M$5</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -620,7 +626,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>zone10!$A$6</c:f>
+              <c:f>zone12!$A$6</c:f>
             </c:strRef>
           </c:tx>
           <c:spPr>
@@ -635,22 +641,22 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>zone10!$B$1:$M$1</c:f>
+              <c:f>zone12!$B$1:$M$1</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>zone10!$B$6:$M$6</c:f>
+              <c:f>zone12!$B$6:$M$6</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1441222995"/>
-        <c:axId val="1683762011"/>
+        <c:axId val="585472597"/>
+        <c:axId val="89660641"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1441222995"/>
+        <c:axId val="585472597"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -687,7 +693,11 @@
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:spPr/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
@@ -702,10 +712,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1683762011"/>
+        <c:crossAx val="89660641"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1683762011"/>
+        <c:axId val="89660641"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -764,7 +774,9 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
-          <a:ln/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
         </c:spPr>
         <c:txPr>
           <a:bodyPr/>
@@ -780,7 +792,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1441222995"/>
+        <c:crossAx val="585472597"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -995,11 +1007,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="835600814"/>
-        <c:axId val="1293527587"/>
+        <c:axId val="431414676"/>
+        <c:axId val="342590526"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="835600814"/>
+        <c:axId val="431414676"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1036,7 +1048,11 @@
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:spPr/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
@@ -1051,10 +1067,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1293527587"/>
+        <c:crossAx val="342590526"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1293527587"/>
+        <c:axId val="342590526"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1113,7 +1129,9 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
-          <a:ln/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
         </c:spPr>
         <c:txPr>
           <a:bodyPr/>
@@ -1129,7 +1147,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="835600814"/>
+        <c:crossAx val="431414676"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1194,7 +1212,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>zone12!$A$2</c:f>
+              <c:f>zone10!$A$2</c:f>
             </c:strRef>
           </c:tx>
           <c:spPr>
@@ -1209,12 +1227,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>zone12!$B$1:$M$1</c:f>
+              <c:f>zone10!$B$1:$M$1</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>zone12!$B$2:$M$2</c:f>
+              <c:f>zone10!$B$2:$M$2</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -1225,7 +1243,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>zone12!$A$3</c:f>
+              <c:f>zone10!$A$3</c:f>
             </c:strRef>
           </c:tx>
           <c:spPr>
@@ -1240,12 +1258,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>zone12!$B$1:$M$1</c:f>
+              <c:f>zone10!$B$1:$M$1</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>zone12!$B$3:$M$3</c:f>
+              <c:f>zone10!$B$3:$M$3</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -1256,7 +1274,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>zone12!$A$4</c:f>
+              <c:f>zone10!$A$4</c:f>
             </c:strRef>
           </c:tx>
           <c:spPr>
@@ -1271,12 +1289,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>zone12!$B$1:$M$1</c:f>
+              <c:f>zone10!$B$1:$M$1</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>zone12!$B$4:$M$4</c:f>
+              <c:f>zone10!$B$4:$M$4</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -1287,7 +1305,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>zone12!$A$5</c:f>
+              <c:f>zone10!$A$5</c:f>
             </c:strRef>
           </c:tx>
           <c:spPr>
@@ -1302,12 +1320,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>zone12!$B$1:$M$1</c:f>
+              <c:f>zone10!$B$1:$M$1</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>zone12!$B$5:$M$5</c:f>
+              <c:f>zone10!$B$5:$M$5</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -1318,7 +1336,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>zone12!$A$6</c:f>
+              <c:f>zone10!$A$6</c:f>
             </c:strRef>
           </c:tx>
           <c:spPr>
@@ -1333,22 +1351,22 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>zone12!$B$1:$M$1</c:f>
+              <c:f>zone10!$B$1:$M$1</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>zone12!$B$6:$M$6</c:f>
+              <c:f>zone10!$B$6:$M$6</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1749077516"/>
-        <c:axId val="679138586"/>
+        <c:axId val="1842185454"/>
+        <c:axId val="2112324606"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1749077516"/>
+        <c:axId val="1842185454"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1385,7 +1403,11 @@
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:spPr/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
@@ -1400,10 +1422,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="679138586"/>
+        <c:crossAx val="2112324606"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="679138586"/>
+        <c:axId val="2112324606"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1462,7 +1484,9 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
-          <a:ln/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
         </c:spPr>
         <c:txPr>
           <a:bodyPr/>
@@ -1478,7 +1502,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1749077516"/>
+        <c:crossAx val="1842185454"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1693,11 +1717,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="682938531"/>
-        <c:axId val="1089141350"/>
+        <c:axId val="283698835"/>
+        <c:axId val="1590522382"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="682938531"/>
+        <c:axId val="283698835"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1734,7 +1758,11 @@
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:spPr/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
@@ -1749,10 +1777,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1089141350"/>
+        <c:crossAx val="1590522382"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1089141350"/>
+        <c:axId val="1590522382"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1811,7 +1839,9 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
-          <a:ln/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
         </c:spPr>
         <c:txPr>
           <a:bodyPr/>
@@ -1827,7 +1857,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="682938531"/>
+        <c:crossAx val="283698835"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2042,11 +2072,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1336831463"/>
-        <c:axId val="1440631184"/>
+        <c:axId val="1387015992"/>
+        <c:axId val="933521930"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1336831463"/>
+        <c:axId val="1387015992"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2083,7 +2113,11 @@
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:spPr/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
@@ -2098,10 +2132,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1440631184"/>
+        <c:crossAx val="933521930"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1440631184"/>
+        <c:axId val="933521930"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2160,7 +2194,9 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
-          <a:ln/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
         </c:spPr>
         <c:txPr>
           <a:bodyPr/>
@@ -2176,7 +2212,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1336831463"/>
+        <c:crossAx val="1387015992"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2391,11 +2427,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1586952318"/>
-        <c:axId val="1859944321"/>
+        <c:axId val="495414529"/>
+        <c:axId val="1474630791"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1586952318"/>
+        <c:axId val="495414529"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2432,7 +2468,11 @@
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:spPr/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
@@ -2447,10 +2487,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1859944321"/>
+        <c:crossAx val="1474630791"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1859944321"/>
+        <c:axId val="1474630791"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2509,7 +2549,9 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
-          <a:ln/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
         </c:spPr>
         <c:txPr>
           <a:bodyPr/>
@@ -2525,7 +2567,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1586952318"/>
+        <c:crossAx val="495414529"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2740,11 +2782,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1558810494"/>
-        <c:axId val="832946874"/>
+        <c:axId val="1483085159"/>
+        <c:axId val="843254706"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1558810494"/>
+        <c:axId val="1483085159"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2781,7 +2823,11 @@
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:spPr/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
@@ -2796,10 +2842,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="832946874"/>
+        <c:crossAx val="843254706"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="832946874"/>
+        <c:axId val="843254706"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2858,7 +2904,9 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
-          <a:ln/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
         </c:spPr>
         <c:txPr>
           <a:bodyPr/>
@@ -2874,7 +2922,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1558810494"/>
+        <c:crossAx val="1483085159"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -3089,11 +3137,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="130867082"/>
-        <c:axId val="364541478"/>
+        <c:axId val="167395280"/>
+        <c:axId val="2094745528"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="130867082"/>
+        <c:axId val="167395280"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3130,7 +3178,11 @@
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:spPr/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
@@ -3145,10 +3197,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="364541478"/>
+        <c:crossAx val="2094745528"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="364541478"/>
+        <c:axId val="2094745528"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3207,7 +3259,9 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
-          <a:ln/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
         </c:spPr>
         <c:txPr>
           <a:bodyPr/>
@@ -3223,7 +3277,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="130867082"/>
+        <c:crossAx val="167395280"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -3438,11 +3492,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="141967401"/>
-        <c:axId val="441993203"/>
+        <c:axId val="1153976577"/>
+        <c:axId val="1440930859"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="141967401"/>
+        <c:axId val="1153976577"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3479,7 +3533,11 @@
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:spPr/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
@@ -3494,10 +3552,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="441993203"/>
+        <c:crossAx val="1440930859"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="441993203"/>
+        <c:axId val="1440930859"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3556,7 +3614,9 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
-          <a:ln/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
         </c:spPr>
         <c:txPr>
           <a:bodyPr/>
@@ -3572,7 +3632,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="141967401"/>
+        <c:crossAx val="1153976577"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -3787,11 +3847,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1901319283"/>
-        <c:axId val="855076818"/>
+        <c:axId val="2121794655"/>
+        <c:axId val="1725883459"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1901319283"/>
+        <c:axId val="2121794655"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3828,7 +3888,11 @@
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:spPr/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
@@ -3843,10 +3907,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="855076818"/>
+        <c:crossAx val="1725883459"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="855076818"/>
+        <c:axId val="1725883459"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3905,7 +3969,9 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
-          <a:ln/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
         </c:spPr>
         <c:txPr>
           <a:bodyPr/>
@@ -3921,7 +3987,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1901319283"/>
+        <c:crossAx val="2121794655"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -4136,11 +4202,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1082493283"/>
-        <c:axId val="566247041"/>
+        <c:axId val="1009730952"/>
+        <c:axId val="1913766692"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1082493283"/>
+        <c:axId val="1009730952"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4177,7 +4243,11 @@
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:spPr/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
@@ -4192,10 +4262,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="566247041"/>
+        <c:crossAx val="1913766692"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="566247041"/>
+        <c:axId val="1913766692"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4254,7 +4324,9 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
-          <a:ln/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
         </c:spPr>
         <c:txPr>
           <a:bodyPr/>
@@ -4270,7 +4342,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1082493283"/>
+        <c:crossAx val="1009730952"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -4308,7 +4380,7 @@
     <xdr:ext cx="6362700" cy="3924300"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="1" name="Chart 1" title="Chart"/>
+        <xdr:cNvPr id="3" name="Chart 3" title="Chart"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -4338,7 +4410,7 @@
     <xdr:ext cx="6362700" cy="3924300"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="10" name="Chart 10" title="Chart"/>
+        <xdr:cNvPr id="9" name="Chart 9" title="Chart"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -4368,7 +4440,7 @@
     <xdr:ext cx="6362700" cy="3924300"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="11" name="Chart 11" title="Chart"/>
+        <xdr:cNvPr id="10" name="Chart 10" title="Chart"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -4428,7 +4500,7 @@
     <xdr:ext cx="6362700" cy="3924300"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 2" title="Chart"/>
+        <xdr:cNvPr id="4" name="Chart 4" title="Chart"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -4458,7 +4530,7 @@
     <xdr:ext cx="6362700" cy="3924300"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 3" title="Chart"/>
+        <xdr:cNvPr id="2" name="Chart 2" title="Chart"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -4488,7 +4560,7 @@
     <xdr:ext cx="6362700" cy="3924300"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 4" title="Chart"/>
+        <xdr:cNvPr id="1" name="Chart 1" title="Chart"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -4548,7 +4620,7 @@
     <xdr:ext cx="6362700" cy="3924300"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="6" name="Chart 6" title="Chart"/>
+        <xdr:cNvPr id="8" name="Chart 8" title="Chart"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -4578,7 +4650,7 @@
     <xdr:ext cx="6362700" cy="3924300"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="7" name="Chart 7" title="Chart"/>
+        <xdr:cNvPr id="6" name="Chart 6" title="Chart"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -4608,7 +4680,7 @@
     <xdr:ext cx="6362700" cy="3924300"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="8" name="Chart 8" title="Chart"/>
+        <xdr:cNvPr id="7" name="Chart 7" title="Chart"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -4638,7 +4710,7 @@
     <xdr:ext cx="6362700" cy="3924300"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="9" name="Chart 9" title="Chart"/>
+        <xdr:cNvPr id="11" name="Chart 11" title="Chart"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -5210,40 +5282,40 @@
         <v>1</v>
       </c>
       <c r="B2" s="4">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="C2" s="4">
         <v>5.0</v>
       </c>
       <c r="D2" s="4">
-        <v>11.0</v>
+        <v>12.0</v>
       </c>
       <c r="E2" s="4">
-        <v>19.0</v>
+        <v>21.0</v>
       </c>
       <c r="F2" s="4">
-        <v>36.0</v>
+        <v>37.0</v>
       </c>
       <c r="G2" s="4">
         <v>52.0</v>
       </c>
       <c r="H2" s="4">
-        <v>67.0</v>
+        <v>66.0</v>
       </c>
       <c r="I2" s="4">
-        <v>81.0</v>
+        <v>80.0</v>
       </c>
       <c r="J2" s="4">
-        <v>88.0</v>
+        <v>87.0</v>
       </c>
       <c r="K2" s="4">
-        <v>95.0</v>
+        <v>93.0</v>
       </c>
       <c r="L2" s="4">
-        <v>100.0</v>
+        <v>99.0</v>
       </c>
       <c r="M2" s="4">
-        <v>105.0</v>
+        <v>104.0</v>
       </c>
     </row>
     <row r="3">
@@ -5251,7 +5323,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="4">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="C3" s="4">
         <v>5.0</v>
@@ -5260,7 +5332,7 @@
         <v>11.0</v>
       </c>
       <c r="E3" s="4">
-        <v>19.0</v>
+        <v>18.0</v>
       </c>
       <c r="F3" s="4">
         <v>34.0</v>
@@ -5269,19 +5341,19 @@
         <v>49.0</v>
       </c>
       <c r="H3" s="4">
-        <v>64.0</v>
+        <v>62.0</v>
       </c>
       <c r="I3" s="4">
-        <v>77.0</v>
+        <v>76.0</v>
       </c>
       <c r="J3" s="4">
-        <v>84.0</v>
+        <v>82.0</v>
       </c>
       <c r="K3" s="4">
-        <v>90.0</v>
+        <v>88.0</v>
       </c>
       <c r="L3" s="4">
-        <v>95.0</v>
+        <v>93.0</v>
       </c>
       <c r="M3" s="4">
         <v>99.0</v>
@@ -5310,22 +5382,22 @@
         <v>40.0</v>
       </c>
       <c r="H4" s="4">
-        <v>52.0</v>
+        <v>51.0</v>
       </c>
       <c r="I4" s="4">
-        <v>63.0</v>
+        <v>62.0</v>
       </c>
       <c r="J4" s="4">
-        <v>68.0</v>
+        <v>67.0</v>
       </c>
       <c r="K4" s="4">
-        <v>73.0</v>
+        <v>71.0</v>
       </c>
       <c r="L4" s="4">
+        <v>74.0</v>
+      </c>
+      <c r="M4" s="4">
         <v>77.0</v>
-      </c>
-      <c r="M4" s="4">
-        <v>81.0</v>
       </c>
     </row>
     <row r="5">
@@ -5354,19 +5426,19 @@
         <v>63.0</v>
       </c>
       <c r="I5" s="4">
-        <v>76.0</v>
+        <v>77.0</v>
       </c>
       <c r="J5" s="4">
-        <v>80.0</v>
+        <v>83.0</v>
       </c>
       <c r="K5" s="4">
-        <v>81.0</v>
+        <v>88.0</v>
       </c>
       <c r="L5" s="4">
-        <v>82.0</v>
+        <v>88.0</v>
       </c>
       <c r="M5" s="4">
-        <v>82.0</v>
+        <v>89.0</v>
       </c>
     </row>
     <row r="6">
@@ -5377,7 +5449,7 @@
         <v>0.0</v>
       </c>
       <c r="C6" s="4">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="D6" s="4">
         <v>9.0</v>
@@ -5389,25 +5461,25 @@
         <v>29.0</v>
       </c>
       <c r="G6" s="4">
-        <v>41.0</v>
+        <v>40.0</v>
       </c>
       <c r="H6" s="4">
         <v>51.0</v>
       </c>
       <c r="I6" s="4">
-        <v>60.0</v>
+        <v>61.0</v>
       </c>
       <c r="J6" s="4">
-        <v>62.0</v>
+        <v>64.0</v>
       </c>
       <c r="K6" s="4">
-        <v>63.0</v>
+        <v>66.0</v>
       </c>
       <c r="L6" s="4">
-        <v>63.0</v>
+        <v>67.0</v>
       </c>
       <c r="M6" s="4">
-        <v>63.0</v>
+        <v>67.0</v>
       </c>
     </row>
     <row r="7">
@@ -5783,40 +5855,40 @@
         <v>1</v>
       </c>
       <c r="B2" s="4">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="C2" s="4">
         <v>5.0</v>
       </c>
       <c r="D2" s="4">
-        <v>12.0</v>
+        <v>11.0</v>
       </c>
       <c r="E2" s="4">
-        <v>21.0</v>
+        <v>19.0</v>
       </c>
       <c r="F2" s="4">
-        <v>37.0</v>
+        <v>36.0</v>
       </c>
       <c r="G2" s="4">
         <v>52.0</v>
       </c>
       <c r="H2" s="4">
-        <v>66.0</v>
+        <v>67.0</v>
       </c>
       <c r="I2" s="4">
-        <v>80.0</v>
+        <v>81.0</v>
       </c>
       <c r="J2" s="4">
-        <v>87.0</v>
+        <v>88.0</v>
       </c>
       <c r="K2" s="4">
-        <v>93.0</v>
+        <v>95.0</v>
       </c>
       <c r="L2" s="4">
-        <v>99.0</v>
+        <v>100.0</v>
       </c>
       <c r="M2" s="4">
-        <v>104.0</v>
+        <v>105.0</v>
       </c>
     </row>
     <row r="3">
@@ -5824,7 +5896,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="4">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="C3" s="4">
         <v>5.0</v>
@@ -5833,7 +5905,7 @@
         <v>11.0</v>
       </c>
       <c r="E3" s="4">
-        <v>18.0</v>
+        <v>19.0</v>
       </c>
       <c r="F3" s="4">
         <v>34.0</v>
@@ -5842,19 +5914,19 @@
         <v>49.0</v>
       </c>
       <c r="H3" s="4">
-        <v>62.0</v>
+        <v>64.0</v>
       </c>
       <c r="I3" s="4">
-        <v>76.0</v>
+        <v>77.0</v>
       </c>
       <c r="J3" s="4">
-        <v>82.0</v>
+        <v>84.0</v>
       </c>
       <c r="K3" s="4">
-        <v>88.0</v>
+        <v>90.0</v>
       </c>
       <c r="L3" s="4">
-        <v>93.0</v>
+        <v>95.0</v>
       </c>
       <c r="M3" s="4">
         <v>99.0</v>
@@ -5883,22 +5955,22 @@
         <v>40.0</v>
       </c>
       <c r="H4" s="4">
-        <v>51.0</v>
+        <v>52.0</v>
       </c>
       <c r="I4" s="4">
-        <v>62.0</v>
+        <v>63.0</v>
       </c>
       <c r="J4" s="4">
-        <v>67.0</v>
+        <v>68.0</v>
       </c>
       <c r="K4" s="4">
-        <v>71.0</v>
+        <v>73.0</v>
       </c>
       <c r="L4" s="4">
-        <v>74.0</v>
+        <v>77.0</v>
       </c>
       <c r="M4" s="4">
-        <v>77.0</v>
+        <v>81.0</v>
       </c>
     </row>
     <row r="5">
@@ -5927,19 +5999,19 @@
         <v>63.0</v>
       </c>
       <c r="I5" s="4">
-        <v>77.0</v>
+        <v>76.0</v>
       </c>
       <c r="J5" s="4">
-        <v>83.0</v>
+        <v>80.0</v>
       </c>
       <c r="K5" s="4">
-        <v>88.0</v>
+        <v>81.0</v>
       </c>
       <c r="L5" s="4">
-        <v>88.0</v>
+        <v>82.0</v>
       </c>
       <c r="M5" s="4">
-        <v>89.0</v>
+        <v>82.0</v>
       </c>
     </row>
     <row r="6">
@@ -5950,7 +6022,7 @@
         <v>0.0</v>
       </c>
       <c r="C6" s="4">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="D6" s="4">
         <v>9.0</v>
@@ -5962,25 +6034,25 @@
         <v>29.0</v>
       </c>
       <c r="G6" s="4">
-        <v>40.0</v>
+        <v>41.0</v>
       </c>
       <c r="H6" s="4">
         <v>51.0</v>
       </c>
       <c r="I6" s="4">
-        <v>61.0</v>
+        <v>60.0</v>
       </c>
       <c r="J6" s="4">
-        <v>64.0</v>
+        <v>62.0</v>
       </c>
       <c r="K6" s="4">
-        <v>66.0</v>
+        <v>63.0</v>
       </c>
       <c r="L6" s="4">
-        <v>67.0</v>
+        <v>63.0</v>
       </c>
       <c r="M6" s="4">
-        <v>67.0</v>
+        <v>63.0</v>
       </c>
     </row>
     <row r="7">
@@ -6932,37 +7004,37 @@
         <v>0.0</v>
       </c>
       <c r="C2" s="4">
-        <v>5.0</v>
+        <v>3.0</v>
       </c>
       <c r="D2" s="4">
-        <v>12.0</v>
+        <v>8.0</v>
       </c>
       <c r="E2" s="4">
-        <v>19.0</v>
+        <v>15.0</v>
       </c>
       <c r="F2" s="4">
-        <v>36.0</v>
+        <v>31.0</v>
       </c>
       <c r="G2" s="4">
-        <v>51.0</v>
+        <v>46.0</v>
       </c>
       <c r="H2" s="4">
-        <v>65.0</v>
+        <v>60.0</v>
       </c>
       <c r="I2" s="4">
-        <v>79.0</v>
+        <v>73.0</v>
       </c>
       <c r="J2" s="4">
+        <v>80.0</v>
+      </c>
+      <c r="K2" s="4">
         <v>86.0</v>
       </c>
-      <c r="K2" s="4">
-        <v>92.0</v>
-      </c>
       <c r="L2" s="4">
-        <v>98.0</v>
+        <v>91.0</v>
       </c>
       <c r="M2" s="4">
-        <v>102.0</v>
+        <v>94.0</v>
       </c>
     </row>
     <row r="3">
@@ -6970,40 +7042,40 @@
         <v>2</v>
       </c>
       <c r="B3" s="4">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="C3" s="4">
-        <v>5.0</v>
+        <v>3.0</v>
       </c>
       <c r="D3" s="4">
-        <v>11.0</v>
+        <v>8.0</v>
       </c>
       <c r="E3" s="4">
-        <v>18.0</v>
+        <v>15.0</v>
       </c>
       <c r="F3" s="4">
-        <v>34.0</v>
+        <v>30.0</v>
       </c>
       <c r="G3" s="4">
-        <v>48.0</v>
+        <v>44.0</v>
       </c>
       <c r="H3" s="4">
-        <v>62.0</v>
+        <v>57.0</v>
       </c>
       <c r="I3" s="4">
+        <v>69.0</v>
+      </c>
+      <c r="J3" s="4">
+        <v>72.0</v>
+      </c>
+      <c r="K3" s="4">
+        <v>74.0</v>
+      </c>
+      <c r="L3" s="4">
         <v>75.0</v>
       </c>
-      <c r="J3" s="4">
-        <v>81.0</v>
-      </c>
-      <c r="K3" s="4">
-        <v>87.0</v>
-      </c>
-      <c r="L3" s="4">
-        <v>92.0</v>
-      </c>
       <c r="M3" s="4">
-        <v>96.0</v>
+        <v>76.0</v>
       </c>
     </row>
     <row r="4">
@@ -7014,31 +7086,31 @@
         <v>0.0</v>
       </c>
       <c r="C4" s="4">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="D4" s="4">
-        <v>9.0</v>
+        <v>7.0</v>
       </c>
       <c r="E4" s="4">
-        <v>15.0</v>
+        <v>13.0</v>
       </c>
       <c r="F4" s="4">
-        <v>28.0</v>
+        <v>26.0</v>
       </c>
       <c r="G4" s="4">
-        <v>40.0</v>
+        <v>38.0</v>
       </c>
       <c r="H4" s="4">
-        <v>51.0</v>
+        <v>50.0</v>
       </c>
       <c r="I4" s="4">
-        <v>62.0</v>
+        <v>61.0</v>
       </c>
       <c r="J4" s="4">
-        <v>67.0</v>
+        <v>66.0</v>
       </c>
       <c r="K4" s="4">
-        <v>72.0</v>
+        <v>71.0</v>
       </c>
       <c r="L4" s="4">
         <v>76.0</v>
@@ -7052,31 +7124,31 @@
         <v>4</v>
       </c>
       <c r="B5" s="4">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="C5" s="4">
-        <v>5.0</v>
+        <v>3.0</v>
       </c>
       <c r="D5" s="4">
-        <v>11.0</v>
+        <v>8.0</v>
       </c>
       <c r="E5" s="4">
-        <v>18.0</v>
+        <v>15.0</v>
       </c>
       <c r="F5" s="4">
-        <v>33.0</v>
+        <v>30.0</v>
       </c>
       <c r="G5" s="4">
-        <v>48.0</v>
+        <v>45.0</v>
       </c>
       <c r="H5" s="4">
-        <v>61.0</v>
+        <v>59.0</v>
       </c>
       <c r="I5" s="4">
-        <v>74.0</v>
+        <v>73.0</v>
       </c>
       <c r="J5" s="4">
-        <v>78.0</v>
+        <v>77.0</v>
       </c>
       <c r="K5" s="4">
         <v>80.0</v>
@@ -7096,37 +7168,37 @@
         <v>0.0</v>
       </c>
       <c r="C6" s="4">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="D6" s="4">
-        <v>8.0</v>
+        <v>7.0</v>
       </c>
       <c r="E6" s="4">
         <v>14.0</v>
       </c>
       <c r="F6" s="4">
-        <v>25.0</v>
+        <v>30.0</v>
       </c>
       <c r="G6" s="4">
-        <v>37.0</v>
+        <v>44.0</v>
       </c>
       <c r="H6" s="4">
-        <v>46.0</v>
+        <v>57.0</v>
       </c>
       <c r="I6" s="4">
-        <v>54.0</v>
+        <v>63.0</v>
       </c>
       <c r="J6" s="4">
-        <v>57.0</v>
+        <v>63.0</v>
       </c>
       <c r="K6" s="4">
-        <v>59.0</v>
+        <v>63.0</v>
       </c>
       <c r="L6" s="4">
-        <v>59.0</v>
+        <v>63.0</v>
       </c>
       <c r="M6" s="4">
-        <v>60.0</v>
+        <v>63.0</v>
       </c>
     </row>
     <row r="7">

</xml_diff>